<commit_message>
03: gateway RSSI/SNR, animation import, statistics table
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/statistical_description.xlsx
+++ b/statistical_description.xlsx
@@ -520,10 +520,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>37.34575783424336</v>
+        <v>37.34575783424334</v>
       </c>
       <c r="D3" t="n">
-        <v>6.482859032778124</v>
+        <v>6.482859032778125</v>
       </c>
       <c r="E3" t="n">
         <v>13.96</v>
@@ -556,7 +556,7 @@
         <v>2.064765594994014</v>
       </c>
       <c r="D4" t="n">
-        <v>2.53455505977305</v>
+        <v>2.534555059773049</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -589,7 +589,7 @@
         <v>322.6969035089136</v>
       </c>
       <c r="D5" t="n">
-        <v>8.494172126422965</v>
+        <v>8.494172126422963</v>
       </c>
       <c r="E5" t="n">
         <v>286.91</v>
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23.74074421510393</v>
+        <v>23.74074421510394</v>
       </c>
       <c r="D6" t="n">
-        <v>3.711613999081814</v>
+        <v>3.711613999081815</v>
       </c>
       <c r="E6" t="n">
         <v>13.74</v>
@@ -652,22 +652,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-75.11641989524432</v>
+        <v>-69.57774435514361</v>
       </c>
       <c r="D7" t="n">
-        <v>22.05405367114712</v>
+        <v>17.32955813944539</v>
       </c>
       <c r="E7" t="n">
         <v>-128</v>
       </c>
       <c r="F7" t="n">
-        <v>-91</v>
+        <v>-84</v>
       </c>
       <c r="G7" t="n">
-        <v>-71</v>
+        <v>-68</v>
       </c>
       <c r="H7" t="n">
-        <v>-57</v>
+        <v>-54</v>
       </c>
       <c r="I7" t="n">
         <v>-28</v>
@@ -685,22 +685,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7.9713349218551</v>
+        <v>9.898053048760337</v>
       </c>
       <c r="D8" t="n">
-        <v>6.526893324470904</v>
+        <v>2.134499543767664</v>
       </c>
       <c r="E8" t="n">
-        <v>-24.5</v>
+        <v>-20.5</v>
       </c>
       <c r="F8" t="n">
-        <v>8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="H8" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="I8" t="n">
         <v>25.2</v>
@@ -721,7 +721,7 @@
         <v>9.112710158057105</v>
       </c>
       <c r="D9" t="n">
-        <v>1.601501744710999</v>
+        <v>1.601501744710998</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>867.8228457262176</v>
+        <v>867.8228457262185</v>
       </c>
       <c r="D10" t="n">
         <v>0.4610641877304697</v>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.4718851948034393</v>
+        <v>0.4718851948034395</v>
       </c>
       <c r="D11" t="n">
         <v>0.5333773730009826</v>
@@ -820,7 +820,7 @@
         <v>22.74755277862356</v>
       </c>
       <c r="D12" t="n">
-        <v>12.2962608807795</v>
+        <v>12.29626088077951</v>
       </c>
       <c r="E12" t="n">
         <v>8</v>
@@ -849,7 +849,7 @@
         <v>0.6716223689530927</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7499756835717255</v>
+        <v>0.7499756835717246</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -878,7 +878,7 @@
         <v>1.831174106852896</v>
       </c>
       <c r="D14" t="n">
-        <v>1.669175369014386</v>
+        <v>1.669175369014384</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -908,22 +908,22 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>92.3764198952438</v>
+        <v>86.8377443551436</v>
       </c>
       <c r="D15" t="n">
-        <v>22.05405367114713</v>
+        <v>17.32955813944539</v>
       </c>
       <c r="E15" t="n">
         <v>45.26</v>
       </c>
       <c r="F15" t="n">
-        <v>74.25999999999999</v>
+        <v>71.25999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>88.25999999999999</v>
+        <v>85.25999999999999</v>
       </c>
       <c r="H15" t="n">
-        <v>108.26</v>
+        <v>101.26</v>
       </c>
       <c r="I15" t="n">
         <v>145.26</v>
@@ -941,22 +941,22 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-84.54313662807775</v>
+        <v>-79.94815294814909</v>
       </c>
       <c r="D16" t="n">
-        <v>19.91707498201135</v>
+        <v>16.92257286785275</v>
       </c>
       <c r="E16" t="n">
         <v>-141.2123840191425</v>
       </c>
       <c r="F16" t="n">
-        <v>-100.4668316388797</v>
+        <v>-94.23249407632485</v>
       </c>
       <c r="G16" t="n">
-        <v>-82.21081852649533</v>
+        <v>-78.59612087980607</v>
       </c>
       <c r="H16" t="n">
-        <v>-68.5175485570292</v>
+        <v>-65.33195619988427</v>
       </c>
       <c r="I16" t="n">
         <v>-33.14609373817283</v>
@@ -974,22 +974,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-76.57180170622264</v>
+        <v>-70.05009989938874</v>
       </c>
       <c r="D17" t="n">
-        <v>24.27898143112502</v>
+        <v>17.42831987802841</v>
       </c>
       <c r="E17" t="n">
-        <v>-146.5153820769794</v>
+        <v>-143.3292134201546</v>
       </c>
       <c r="F17" t="n">
-        <v>-91.2778545523916</v>
+        <v>-84.3175485570292</v>
       </c>
       <c r="G17" t="n">
-        <v>-70.79009749652566</v>
+        <v>-68.33195619988427</v>
       </c>
       <c r="H17" t="n">
-        <v>-57.75746206410165</v>
+        <v>-54.5149694202523</v>
       </c>
       <c r="I17" t="n">
         <v>-28.39612087980607</v>

</xml_diff>

<commit_message>
03: restore pressure to hPa, fix savefig line
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/statistical_description.xlsx
+++ b/statistical_description.xlsx
@@ -586,25 +586,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>322.6969035089136</v>
+        <v>978.0569035089135</v>
       </c>
       <c r="D5" t="n">
         <v>8.494172126422963</v>
       </c>
       <c r="E5" t="n">
-        <v>286.91</v>
+        <v>942.27</v>
       </c>
       <c r="F5" t="n">
-        <v>317.8</v>
+        <v>973.16</v>
       </c>
       <c r="G5" t="n">
-        <v>323.21</v>
+        <v>978.5700000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>328.4</v>
+        <v>983.76</v>
       </c>
       <c r="I5" t="n">
-        <v>347.57</v>
+        <v>1002.93</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
03: path loss from the per-uplink transmit power
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/statistical_description.xlsx
+++ b/statistical_description.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,10 +520,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>37.34575783424334</v>
+        <v>37.34575783424336</v>
       </c>
       <c r="D3" t="n">
-        <v>6.482859032778125</v>
+        <v>6.482859032778124</v>
       </c>
       <c r="E3" t="n">
         <v>13.96</v>
@@ -556,7 +556,7 @@
         <v>2.064765594994014</v>
       </c>
       <c r="D4" t="n">
-        <v>2.534555059773049</v>
+        <v>2.53455505977305</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>978.0569035089135</v>
+        <v>978.0569035089127</v>
       </c>
       <c r="D5" t="n">
-        <v>8.494172126422963</v>
+        <v>8.494172126422969</v>
       </c>
       <c r="E5" t="n">
         <v>942.27</v>
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23.74074421510394</v>
+        <v>23.74074421510393</v>
       </c>
       <c r="D6" t="n">
-        <v>3.711613999081815</v>
+        <v>3.711613999081814</v>
       </c>
       <c r="E6" t="n">
         <v>13.74</v>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9.898053048760337</v>
+        <v>9.898053048760341</v>
       </c>
       <c r="D8" t="n">
         <v>2.134499543767664</v>
@@ -721,7 +721,7 @@
         <v>9.112710158057105</v>
       </c>
       <c r="D9" t="n">
-        <v>1.601501744710998</v>
+        <v>1.601501744710999</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>867.8228457262185</v>
+        <v>867.8228457262176</v>
       </c>
       <c r="D10" t="n">
         <v>0.4610641877304697</v>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.4718851948034395</v>
+        <v>0.4718851948034393</v>
       </c>
       <c r="D11" t="n">
         <v>0.5333773730009826</v>
@@ -808,77 +808,81 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>distance</t>
+          <t>tx_power</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>dBm</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>22.74755277862356</v>
+        <v>13.32406793838705</v>
       </c>
       <c r="D12" t="n">
-        <v>12.29626088077951</v>
+        <v>0.9744108006180645</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G12" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="H12" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="I12" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>c_walls</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>distance</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="C13" t="n">
-        <v>0.6716223689530927</v>
+        <v>22.74755277862356</v>
       </c>
       <c r="D13" t="n">
-        <v>0.7499756835717246</v>
+        <v>12.2962608807795</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>w_walls</t>
+          <t>c_walls</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>1.831174106852896</v>
+        <v>0.6716223689530927</v>
       </c>
       <c r="D14" t="n">
-        <v>1.669175369014384</v>
+        <v>0.7499756835717255</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -887,52 +891,48 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
         <v>2</v>
-      </c>
-      <c r="H14" t="n">
-        <v>2</v>
-      </c>
-      <c r="I14" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>exp_pl</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>dB</t>
-        </is>
-      </c>
+          <t>w_walls</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
-        <v>86.8377443551436</v>
+        <v>1.831174106852896</v>
       </c>
       <c r="D15" t="n">
-        <v>17.32955813944539</v>
+        <v>1.669175369014386</v>
       </c>
       <c r="E15" t="n">
-        <v>45.26</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>71.25999999999999</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>85.25999999999999</v>
+        <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>101.26</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>145.26</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>n_power</t>
+          <t>exp_pl</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -941,57 +941,90 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-79.94815294814909</v>
+        <v>86.16181229353025</v>
       </c>
       <c r="D16" t="n">
-        <v>16.92257286785275</v>
+        <v>17.35913709730849</v>
       </c>
       <c r="E16" t="n">
-        <v>-141.2123840191425</v>
+        <v>45.26</v>
       </c>
       <c r="F16" t="n">
-        <v>-94.23249407632485</v>
+        <v>71.25999999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>-78.59612087980607</v>
+        <v>84.25999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>-65.33195619988427</v>
+        <v>100.26</v>
       </c>
       <c r="I16" t="n">
-        <v>-33.14609373817283</v>
+        <v>145.26</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>n_power</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>dB</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>-79.94815294814913</v>
+      </c>
+      <c r="D17" t="n">
+        <v>16.92257286785275</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-141.2123840191425</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-94.23249407632485</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-78.59612087980607</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-65.33195619988427</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-33.14609373817283</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>esp</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>dBm</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>-70.05009989938874</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C18" t="n">
+        <v>-70.05009989938878</v>
+      </c>
+      <c r="D18" t="n">
         <v>17.42831987802841</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>-143.3292134201546</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>-84.3175485570292</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G18" t="n">
         <v>-68.33195619988427</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H18" t="n">
         <v>-54.5149694202523</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I18" t="n">
         <v>-28.39612087980607</v>
       </c>
     </row>

</xml_diff>